<commit_message>
Benchmark results Lenovo - 11.07
</commit_message>
<xml_diff>
--- a/analysis/results/Lenovo/comparison.xlsx
+++ b/analysis/results/Lenovo/comparison.xlsx
@@ -561,16 +561,16 @@
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>2.7422</v>
+        <v>2.833</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>2.9459</v>
+        <v>2.9231</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>2.0174</v>
+        <v>2.2543</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>0.0985</v>
+        <v>0.0997</v>
       </c>
       <c r="G2" s="2" t="inlineStr"/>
       <c r="H2" s="2" t="inlineStr"/>
@@ -593,16 +593,16 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>8.394299999999999</v>
+        <v>8.387700000000001</v>
       </c>
       <c r="D3" t="n">
-        <v>8.180199999999999</v>
+        <v>7.9623</v>
       </c>
       <c r="E3" t="n">
-        <v>9.7723</v>
+        <v>9.567</v>
       </c>
       <c r="F3" t="n">
-        <v>0.1766</v>
+        <v>0.1711</v>
       </c>
       <c r="G3" t="n">
         <v>291</v>
@@ -637,16 +637,16 @@
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>8.317</v>
+        <v>8.3666</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>8.129099999999999</v>
+        <v>8.0433</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>8.625999999999999</v>
+        <v>9.075900000000001</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>0.1905</v>
+        <v>0.1891</v>
       </c>
       <c r="G4" s="2" t="n">
         <v>470</v>
@@ -679,19 +679,19 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>9.072100000000001</v>
+        <v>9.18</v>
       </c>
       <c r="D5" t="n">
-        <v>8.9251</v>
+        <v>8.879799999999999</v>
       </c>
       <c r="E5" t="n">
-        <v>10.914</v>
+        <v>10.6299</v>
       </c>
       <c r="F5" t="n">
-        <v>0.3877</v>
+        <v>0.3889</v>
       </c>
       <c r="G5" t="n">
-        <v>794</v>
+        <v>796</v>
       </c>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr"/>
@@ -721,16 +721,16 @@
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>19.7442</v>
+        <v>19.5439</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>19.3787</v>
+        <v>13.7102</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>21.5837</v>
+        <v>20.8654</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>2.9196</v>
+        <v>2.626</v>
       </c>
       <c r="G6" s="2" t="n">
         <v>4608</v>
@@ -763,19 +763,19 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>88.5681</v>
+        <v>86.7098</v>
       </c>
       <c r="D7" t="n">
-        <v>60.4284</v>
+        <v>60.3683</v>
       </c>
       <c r="E7" t="n">
-        <v>99.6189</v>
+        <v>92.31870000000001</v>
       </c>
       <c r="F7" t="n">
-        <v>16.8149</v>
+        <v>16.5672</v>
       </c>
       <c r="G7" t="n">
-        <v>41230</v>
+        <v>41229</v>
       </c>
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr"/>
@@ -805,19 +805,19 @@
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>586.0857999999999</v>
+        <v>585.8397</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>564.0429</v>
+        <v>560.4565</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>612.1128</v>
+        <v>618.1156</v>
       </c>
       <c r="F8" s="2" t="n">
-        <v>115.6071</v>
+        <v>118.0616</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>407491</v>
+        <v>407488</v>
       </c>
       <c r="H8" s="2" t="inlineStr"/>
       <c r="I8" s="2" t="inlineStr"/>
@@ -847,16 +847,16 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>82.9323</v>
+        <v>5.364</v>
       </c>
       <c r="D9" t="n">
-        <v>81.86190000000001</v>
+        <v>5.7112</v>
       </c>
       <c r="E9" t="n">
-        <v>84.22499999999999</v>
+        <v>4.8636</v>
       </c>
       <c r="F9" t="n">
-        <v>133.6696</v>
+        <v>0.0274</v>
       </c>
       <c r="G9" t="n">
         <v>291</v>
@@ -891,16 +891,16 @@
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>83.1232</v>
+        <v>5.4036</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>82.01739999999999</v>
+        <v>5.5898</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>84.49039999999999</v>
+        <v>5.0444</v>
       </c>
       <c r="F10" s="2" t="n">
-        <v>133.6331</v>
+        <v>0.0283</v>
       </c>
       <c r="G10" s="2" t="n">
         <v>470</v>
@@ -933,19 +933,19 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>82.6178</v>
+        <v>5.6399</v>
       </c>
       <c r="D11" t="n">
-        <v>82.2556</v>
+        <v>5.7949</v>
       </c>
       <c r="E11" t="n">
-        <v>83.8687</v>
+        <v>5.8322</v>
       </c>
       <c r="F11" t="n">
-        <v>133.8036</v>
+        <v>0.2301</v>
       </c>
       <c r="G11" t="n">
-        <v>794</v>
+        <v>796</v>
       </c>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr"/>
@@ -975,16 +975,16 @@
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>83.77760000000001</v>
+        <v>6.5497</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>82.9597</v>
+        <v>7.5062</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>85.28060000000001</v>
+        <v>5.9598</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>135.5946</v>
+        <v>1.8888</v>
       </c>
       <c r="G12" s="2" t="n">
         <v>4608</v>
@@ -1017,19 +1017,19 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>94.2552</v>
+        <v>14.7802</v>
       </c>
       <c r="D13" t="n">
-        <v>88.1232</v>
+        <v>15.7184</v>
       </c>
       <c r="E13" t="n">
-        <v>95.41630000000001</v>
+        <v>14.7675</v>
       </c>
       <c r="F13" t="n">
-        <v>151.078</v>
+        <v>15.5604</v>
       </c>
       <c r="G13" t="n">
-        <v>41230</v>
+        <v>41229</v>
       </c>
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr"/>
@@ -1059,19 +1059,19 @@
         </is>
       </c>
       <c r="C14" s="2" t="n">
-        <v>170.2463</v>
+        <v>59.6684</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>138.0483</v>
+        <v>60.0162</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>175.2074</v>
+        <v>57.2727</v>
       </c>
       <c r="F14" s="2" t="n">
-        <v>258.3526</v>
+        <v>94.6776</v>
       </c>
       <c r="G14" s="2" t="n">
-        <v>407491</v>
+        <v>407488</v>
       </c>
       <c r="H14" s="2" t="inlineStr"/>
       <c r="I14" s="2" t="inlineStr"/>
@@ -1215,13 +1215,13 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>2.7422</v>
+        <v>2.833</v>
       </c>
       <c r="D2" t="n">
-        <v>2.9459</v>
+        <v>2.9231</v>
       </c>
       <c r="E2" t="n">
-        <v>2.0174</v>
+        <v>2.2543</v>
       </c>
       <c r="F2" t="n">
         <v>20</v>
@@ -1277,13 +1277,13 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>77.0326</v>
+        <v>77.03749999999999</v>
       </c>
       <c r="D3" t="n">
-        <v>76.9799</v>
+        <v>77.036</v>
       </c>
       <c r="E3" t="n">
-        <v>77.0335</v>
+        <v>76.80289999999999</v>
       </c>
       <c r="F3" t="n">
         <v>20</v>
@@ -1339,13 +1339,13 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>8.394299999999999</v>
+        <v>8.387700000000001</v>
       </c>
       <c r="D4" t="n">
-        <v>8.180199999999999</v>
+        <v>7.9623</v>
       </c>
       <c r="E4" t="n">
-        <v>9.7723</v>
+        <v>9.567</v>
       </c>
       <c r="F4" t="n">
         <v>20</v>
@@ -1401,13 +1401,13 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>8.317</v>
+        <v>8.3666</v>
       </c>
       <c r="D5" t="n">
-        <v>8.129099999999999</v>
+        <v>8.0433</v>
       </c>
       <c r="E5" t="n">
-        <v>8.625999999999999</v>
+        <v>9.075900000000001</v>
       </c>
       <c r="F5" t="n">
         <v>20</v>
@@ -1463,13 +1463,13 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>9.072100000000001</v>
+        <v>9.18</v>
       </c>
       <c r="D6" t="n">
-        <v>8.9251</v>
+        <v>8.879799999999999</v>
       </c>
       <c r="E6" t="n">
-        <v>10.914</v>
+        <v>10.6299</v>
       </c>
       <c r="F6" t="n">
         <v>20</v>
@@ -1478,7 +1478,7 @@
         <v>65536</v>
       </c>
       <c r="H6" t="n">
-        <v>794</v>
+        <v>796</v>
       </c>
       <c r="I6" t="n">
         <v>0</v>
@@ -1525,13 +1525,13 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>19.7442</v>
+        <v>19.5439</v>
       </c>
       <c r="D7" t="n">
-        <v>19.3787</v>
+        <v>13.7102</v>
       </c>
       <c r="E7" t="n">
-        <v>21.5837</v>
+        <v>20.8654</v>
       </c>
       <c r="F7" t="n">
         <v>20</v>
@@ -1587,13 +1587,13 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>88.5681</v>
+        <v>86.7098</v>
       </c>
       <c r="D8" t="n">
-        <v>60.4284</v>
+        <v>60.3683</v>
       </c>
       <c r="E8" t="n">
-        <v>99.6189</v>
+        <v>92.31870000000001</v>
       </c>
       <c r="F8" t="n">
         <v>20</v>
@@ -1602,7 +1602,7 @@
         <v>10485760</v>
       </c>
       <c r="H8" t="n">
-        <v>41230</v>
+        <v>41229</v>
       </c>
       <c r="I8" t="n">
         <v>0</v>
@@ -1649,13 +1649,13 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>586.0857999999999</v>
+        <v>585.8397</v>
       </c>
       <c r="D9" t="n">
-        <v>564.0429</v>
+        <v>560.4565</v>
       </c>
       <c r="E9" t="n">
-        <v>612.1128</v>
+        <v>618.1156</v>
       </c>
       <c r="F9" t="n">
         <v>20</v>
@@ -1664,7 +1664,7 @@
         <v>104857600</v>
       </c>
       <c r="H9" t="n">
-        <v>407491</v>
+        <v>407488</v>
       </c>
       <c r="I9" t="n">
         <v>0</v>
@@ -1711,13 +1711,13 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>82.9323</v>
+        <v>5.364</v>
       </c>
       <c r="D10" t="n">
-        <v>81.86190000000001</v>
+        <v>5.7112</v>
       </c>
       <c r="E10" t="n">
-        <v>84.22499999999999</v>
+        <v>4.8636</v>
       </c>
       <c r="F10" t="n">
         <v>20</v>
@@ -1773,13 +1773,13 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>83.1232</v>
+        <v>5.4036</v>
       </c>
       <c r="D11" t="n">
-        <v>82.01739999999999</v>
+        <v>5.5898</v>
       </c>
       <c r="E11" t="n">
-        <v>84.49039999999999</v>
+        <v>5.0444</v>
       </c>
       <c r="F11" t="n">
         <v>20</v>
@@ -1835,13 +1835,13 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>82.6178</v>
+        <v>5.6399</v>
       </c>
       <c r="D12" t="n">
-        <v>82.2556</v>
+        <v>5.7949</v>
       </c>
       <c r="E12" t="n">
-        <v>83.8687</v>
+        <v>5.8322</v>
       </c>
       <c r="F12" t="n">
         <v>20</v>
@@ -1897,13 +1897,13 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>83.77760000000001</v>
+        <v>6.5497</v>
       </c>
       <c r="D13" t="n">
-        <v>82.9597</v>
+        <v>7.5062</v>
       </c>
       <c r="E13" t="n">
-        <v>85.28060000000001</v>
+        <v>5.9598</v>
       </c>
       <c r="F13" t="n">
         <v>20</v>
@@ -1959,13 +1959,13 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>94.2552</v>
+        <v>14.7802</v>
       </c>
       <c r="D14" t="n">
-        <v>88.1232</v>
+        <v>15.7184</v>
       </c>
       <c r="E14" t="n">
-        <v>95.41630000000001</v>
+        <v>14.7675</v>
       </c>
       <c r="F14" t="n">
         <v>20</v>
@@ -2021,13 +2021,13 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>170.2463</v>
+        <v>59.6684</v>
       </c>
       <c r="D15" t="n">
-        <v>138.0483</v>
+        <v>60.0162</v>
       </c>
       <c r="E15" t="n">
-        <v>175.2074</v>
+        <v>57.2727</v>
       </c>
       <c r="F15" t="n">
         <v>20</v>
@@ -2222,7 +2222,7 @@
         <v>65536</v>
       </c>
       <c r="H18" t="n">
-        <v>798</v>
+        <v>797</v>
       </c>
       <c r="I18" t="n">
         <v>0</v>
@@ -2284,7 +2284,7 @@
         <v>1048576</v>
       </c>
       <c r="H19" t="n">
-        <v>4610</v>
+        <v>4611</v>
       </c>
       <c r="I19" t="n">
         <v>0</v>
@@ -2545,16 +2545,16 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.09854300000000001</v>
+        <v>0.099689</v>
       </c>
       <c r="D2" t="n">
-        <v>0.09854300000000001</v>
+        <v>0.099689</v>
       </c>
       <c r="E2" t="n">
-        <v>0.09854300000000001</v>
+        <v>0.099689</v>
       </c>
       <c r="F2" t="n">
-        <v>119365</v>
+        <v>119420</v>
       </c>
       <c r="G2" t="n">
         <v>0</v>
@@ -2595,13 +2595,13 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>77.122725</v>
+        <v>77.111504</v>
       </c>
       <c r="D3" t="n">
-        <v>77.122725</v>
+        <v>77.111504</v>
       </c>
       <c r="E3" t="n">
-        <v>77.122725</v>
+        <v>77.111504</v>
       </c>
       <c r="F3" t="n">
         <v>154</v>
@@ -2645,16 +2645,16 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.176609</v>
+        <v>0.171137</v>
       </c>
       <c r="D4" t="n">
-        <v>0.176609</v>
+        <v>0.171137</v>
       </c>
       <c r="E4" t="n">
-        <v>0.176609</v>
+        <v>0.171137</v>
       </c>
       <c r="F4" t="n">
-        <v>69474</v>
+        <v>68869</v>
       </c>
       <c r="G4" t="n">
         <v>100</v>
@@ -2695,16 +2695,16 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.190476</v>
+        <v>0.189071</v>
       </c>
       <c r="D5" t="n">
-        <v>0.190476</v>
+        <v>0.189071</v>
       </c>
       <c r="E5" t="n">
-        <v>0.190476</v>
+        <v>0.189071</v>
       </c>
       <c r="F5" t="n">
-        <v>63584</v>
+        <v>59586</v>
       </c>
       <c r="G5" t="n">
         <v>1024</v>
@@ -2745,16 +2745,16 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0.387728</v>
+        <v>0.388949</v>
       </c>
       <c r="D6" t="n">
-        <v>0.387728</v>
+        <v>0.388949</v>
       </c>
       <c r="E6" t="n">
-        <v>0.387728</v>
+        <v>0.388949</v>
       </c>
       <c r="F6" t="n">
-        <v>30166</v>
+        <v>30224</v>
       </c>
       <c r="G6" t="n">
         <v>65536</v>
@@ -2795,16 +2795,16 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>2.91955</v>
+        <v>2.626024</v>
       </c>
       <c r="D7" t="n">
-        <v>2.91955</v>
+        <v>2.626024</v>
       </c>
       <c r="E7" t="n">
-        <v>2.91955</v>
+        <v>2.626024</v>
       </c>
       <c r="F7" t="n">
-        <v>4838</v>
+        <v>4718</v>
       </c>
       <c r="G7" t="n">
         <v>1048576</v>
@@ -2845,16 +2845,16 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>16.814949</v>
+        <v>16.567166</v>
       </c>
       <c r="D8" t="n">
-        <v>16.814949</v>
+        <v>16.567166</v>
       </c>
       <c r="E8" t="n">
-        <v>16.814949</v>
+        <v>16.567166</v>
       </c>
       <c r="F8" t="n">
-        <v>748</v>
+        <v>752</v>
       </c>
       <c r="G8" t="n">
         <v>10485760</v>
@@ -2895,16 +2895,16 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>115.607094</v>
+        <v>118.061579</v>
       </c>
       <c r="D9" t="n">
-        <v>115.607094</v>
+        <v>118.061579</v>
       </c>
       <c r="E9" t="n">
-        <v>115.607094</v>
+        <v>118.061579</v>
       </c>
       <c r="F9" t="n">
-        <v>100</v>
+        <v>86</v>
       </c>
       <c r="G9" t="n">
         <v>104857600</v>
@@ -2945,16 +2945,16 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>133.669598</v>
+        <v>0.027394</v>
       </c>
       <c r="D10" t="n">
-        <v>133.669598</v>
+        <v>0.027394</v>
       </c>
       <c r="E10" t="n">
-        <v>133.669598</v>
+        <v>0.027394</v>
       </c>
       <c r="F10" t="n">
-        <v>88</v>
+        <v>411091</v>
       </c>
       <c r="G10" t="n">
         <v>100</v>
@@ -2995,16 +2995,16 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>133.633101</v>
+        <v>0.028335</v>
       </c>
       <c r="D11" t="n">
-        <v>133.633101</v>
+        <v>0.028335</v>
       </c>
       <c r="E11" t="n">
-        <v>133.633101</v>
+        <v>0.028335</v>
       </c>
       <c r="F11" t="n">
-        <v>88</v>
+        <v>403280</v>
       </c>
       <c r="G11" t="n">
         <v>1024</v>
@@ -3045,16 +3045,16 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>133.803558</v>
+        <v>0.230105</v>
       </c>
       <c r="D12" t="n">
-        <v>133.803558</v>
+        <v>0.230105</v>
       </c>
       <c r="E12" t="n">
-        <v>133.803558</v>
+        <v>0.230105</v>
       </c>
       <c r="F12" t="n">
-        <v>88</v>
+        <v>49938</v>
       </c>
       <c r="G12" t="n">
         <v>65536</v>
@@ -3095,16 +3095,16 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>135.594568</v>
+        <v>1.888799</v>
       </c>
       <c r="D13" t="n">
-        <v>135.594568</v>
+        <v>1.888799</v>
       </c>
       <c r="E13" t="n">
-        <v>135.594568</v>
+        <v>1.888799</v>
       </c>
       <c r="F13" t="n">
-        <v>87</v>
+        <v>5800</v>
       </c>
       <c r="G13" t="n">
         <v>1048576</v>
@@ -3145,16 +3145,16 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>151.078032</v>
+        <v>15.560368</v>
       </c>
       <c r="D14" t="n">
-        <v>151.078032</v>
+        <v>15.560368</v>
       </c>
       <c r="E14" t="n">
-        <v>151.078032</v>
+        <v>15.560368</v>
       </c>
       <c r="F14" t="n">
-        <v>76</v>
+        <v>746</v>
       </c>
       <c r="G14" t="n">
         <v>10485760</v>
@@ -3195,16 +3195,16 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>258.352589</v>
+        <v>94.677633</v>
       </c>
       <c r="D15" t="n">
-        <v>258.352589</v>
+        <v>94.677633</v>
       </c>
       <c r="E15" t="n">
-        <v>258.352589</v>
+        <v>94.677633</v>
       </c>
       <c r="F15" t="n">
-        <v>45</v>
+        <v>122</v>
       </c>
       <c r="G15" t="n">
         <v>104857600</v>

</xml_diff>